<commit_message>
CAPEX workbook: add summary, per-equipment power, payback and CO2 sheets; fix text cell parsed as formula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4ipyfgS5pJVMtqbwpHHE9
</commit_message>
<xml_diff>
--- a/ccu-thailand-formic-acid/capex/EcoFormic_CAPEX_MEA_Pilot.xlsx
+++ b/ccu-thailand-formic-acid/capex/EcoFormic_CAPEX_MEA_Pilot.xlsx
@@ -7,10 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="งบลงทุน" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ตัดออก" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ขนาดการผลิต" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ข้อควรทราบ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="สรุป" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="งบลงทุน" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ตัดออก" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ขนาดการผลิต" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ข้อควรทราบ" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="การใช้ไฟ" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="คืนทุน" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CO2" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,12 +23,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +68,10 @@
     <font>
       <name val="Arial"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00008000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -122,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,6 +181,41 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,6 +581,315 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>สรุป Skid นำร่อง 100 kW – กรดฟอร์มิกจาก CO₂ บางปะกง (MEA 30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>ทุกค่าดึงจากชีตอื่น แก้ตัวเลขสีน้ำเงินในชีตนั้น ๆ แล้วหน้านี้เปลี่ยนตาม</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>หัวข้อ</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ค่า</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>หน่วย</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>เงินลงทุนรวม (รวมเงินสำรอง)</t>
+        </is>
+      </c>
+      <c r="B5" s="30">
+        <f>'งบลงทุน'!F71</f>
+        <v/>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>บาท</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>ผลผลิตกรด 85%</t>
+        </is>
+      </c>
+      <c r="B6" s="32">
+        <f>'ขนาดการผลิต'!B19</f>
+        <v/>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>เทียบแผนโรงงาน 10,000 ตัน/ปี</t>
+        </is>
+      </c>
+      <c r="B7" s="33">
+        <f>'ขนาดการผลิต'!B21</f>
+        <v/>
+      </c>
+      <c r="C7" s="31" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>กำลังไฟฟ้ารวม</t>
+        </is>
+      </c>
+      <c r="B8" s="32">
+        <f>'การใช้ไฟ'!C43</f>
+        <v/>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>ไฟฟ้าที่ใช้</t>
+        </is>
+      </c>
+      <c r="B9" s="30">
+        <f>'การใช้ไฟ'!E43</f>
+        <v/>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>kWh/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>ค่าไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="B10" s="30">
+        <f>'การใช้ไฟ'!F43</f>
+        <v/>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>ค่าดำเนินการรวม</t>
+        </is>
+      </c>
+      <c r="B11" s="30">
+        <f>'คืนทุน'!$B$18</f>
+        <v/>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>กำไรต่อปี ที่ราคา 39.78 บาท/กก. (S11)</t>
+        </is>
+      </c>
+      <c r="B12" s="30">
+        <f>'คืนทุน'!C25</f>
+        <v/>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>ระยะคืนทุน ที่ราคา 30 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="B13" s="32">
+        <f>'คืนทุน'!B26</f>
+        <v/>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>ระยะคืนทุน ที่ราคา 39.78 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="B14" s="32">
+        <f>'คืนทุน'!C26</f>
+        <v/>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>ระยะคืนทุน ที่ราคา 52.3 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="B15" s="32">
+        <f>'คืนทุน'!D26</f>
+        <v/>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ดักจับ</t>
+        </is>
+      </c>
+      <c r="B16" s="32">
+        <f>'CO2'!$B$4</f>
+        <v/>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>ลด CO₂ สุทธิ ถ้าใช้ไฟโรงไฟฟ้าก๊าซทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B17" s="32">
+        <f>'CO2'!C11</f>
+        <v/>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>ลด CO₂ สุทธิ ถ้า PEM ใช้โซลาร์</t>
+        </is>
+      </c>
+      <c r="B18" s="32">
+        <f>'CO2'!C12</f>
+        <v/>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>ลด CO₂ สุทธิ ถ้าใช้โซลาร์ทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B19" s="32">
+        <f>'CO2'!C13</f>
+        <v/>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ลดได้จากการแทนกรดนำเข้า (นอกบางปะกง)</t>
+        </is>
+      </c>
+      <c r="B20" s="32">
+        <f>'CO2'!B18</f>
+        <v/>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>ตัน CO₂e/ปี</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>ค่าในช่องสีเหลืองของแต่ละชีตเป็นประมาณการ ต้องแทนด้วยสเปกเครื่องและใบเสนอราคาจริง</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -564,6 +919,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1151,6 +1507,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -1357,6 +1714,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
@@ -1778,6 +2136,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
@@ -1976,6 +2335,7 @@
         <v/>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
@@ -2483,6 +2843,7 @@
         <v/>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
@@ -2767,6 +3128,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="E68" s="12" t="inlineStr">
         <is>
@@ -2850,8 +3212,8 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A45:J45"/>
     <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A45:J45"/>
     <mergeCell ref="A59:J59"/>
     <mergeCell ref="A26:J26"/>
     <mergeCell ref="A38:J38"/>
@@ -2862,7 +3224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3029,7 +3391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3204,9 +3566,10 @@
         <f>B3/B4</f>
         <v/>
       </c>
-      <c r="C12" s="22">
-        <f> กำลัง ÷ ไฟฟ้าต่อ kg</f>
-        <v/>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>กำลัง ÷ ไฟฟ้าต่อ kg</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3349,13 +3712,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -3417,6 +3780,2289 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>8. ชีต การใช้ไฟ: พัดลม ปั๊ม MEA และเครื่องอัด คำนวณด้วยสูตรฟิสิกส์จากอัตราไหล; ค่าประสิทธิภาพและความดันตกเป็นประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>9. ไอน้ำสำหรับหอไล่ CO₂ คิดราคา 0 บาท (ไอน้ำเหลือทิ้ง) ต้องตกลงกับ กฟผ.; ความร้อนของหอแยกกรดยังไม่ทราบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>10. คืนทุนแบบง่าย ยังไม่รวมภาษี ดอกเบี้ย ค่าเช่าพื้นที่ และค่าเสื่อมราคา; ราคาขายจริงต้องต่ำกว่าราคา CIF ที่ผู้นำเข้าจ่าย</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>8. ชีต การใช้ไฟ: พัดลม ปั๊ม MEA และเครื่องอัด คำนวณด้วยสูตรฟิสิกส์จากอัตราไหล; ค่าประสิทธิภาพและความดันตกเป็นประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>9. ไอน้ำสำหรับหอไล่ CO₂ คิดราคา 0 บาท (ไอน้ำเหลือทิ้ง) ต้องตกลงกับ กฟผ.; ความร้อนของหอแยกกรดยังไม่ทราบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>10. คืนทุนแบบง่าย ยังไม่รวมภาษี ดอกเบี้ย ค่าเช่าพื้นที่ และค่าเสื่อมราคา; ราคาขายจริงต้องต่ำกว่าราคา CIF ที่ผู้นำเข้าจ่าย</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>การใช้ไฟฟ้าและความร้อนรายอุปกรณ์ (Skid 100 kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>สีน้ำเงิน = แก้ได้ · สีเขียว = ดึงจากชีตอื่น · ช่องสีเหลือง = ประมาณการ ต้องใช้สเปกเครื่องจริง</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ค่าที่ใช้คำนวณ</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ค่า</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ที่มา</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>ค่าไฟ (บาท/kWh)</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>S10 กกพ. ค่าไฟเฉลี่ย ก.ย.–ธ.ค. 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>ชั่วโมงเดินเครื่อง/ปี</t>
+        </is>
+      </c>
+      <c r="B6" s="30">
+        <f>'ขนาดการผลิต'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต (CF 0.65 × 8,760, S04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>ความดันตกผ่านหอทำเย็น+หอดูดซับ+ส่วนล้าง (kPa)</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ – ขึ้นกับแบบหอจริง</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>ประสิทธิภาพพัดลม</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>ความสูงส่งของปั๊ม MEA (m)</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ: ความสูงหอ + ความดันหอไล่ 1.5 bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>ประสิทธิภาพปั๊ม</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>ความหนาแน่น MEA 30% (kg/m³)</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="n">
+        <v>1010</v>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ (ใกล้น้ำ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ความดันขาเข้าเครื่องอัด (bar)</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>S19 ความดันหอไล่</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ความดันขาออก (bar)</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม: เตาทน 50 bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>จำนวนขั้นอัด CO₂</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ (อัตราส่วนความดัน ~33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>k ของ CO₂</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>ค่าคุณสมบัติก๊าซ CO₂</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>H₂ ความดันขาเข้า (bar)</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม: ถังพัก 30–50 bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>H₂ ความดันขาออก (bar)</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>k ของ H₂</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>ค่าคุณสมบัติก๊าซ H₂</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>อุณหภูมิก๊าซเข้าเครื่องอัด (K)</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="n">
+        <v>313.15</v>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>40 °C หลังทำเย็น</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>ประสิทธิภาพเครื่องอัด</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>COP ของ chiller</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>อุปกรณ์</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>ลำดับในงบ</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>กำลังไฟ (kW)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>ชั่วโมง/ปี</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>kWh/ปี</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>ค่าไฟ (บาท/ปี)</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>% ของไฟทั้งหมด</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>วิธีคำนวณ</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>ที่มา</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>พัดลมดูดไอเสีย</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C24" s="41">
+        <f>'ขนาดการผลิต'!B15*(313.15/273.15)/3600*$B$7/$B$8</f>
+        <v/>
+      </c>
+      <c r="D24" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E24" s="42">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="42">
+        <f>E24*$B$5</f>
+        <v/>
+      </c>
+      <c r="G24" s="43">
+        <f>E24/$E$43</f>
+        <v/>
+      </c>
+      <c r="H24" s="31" t="inlineStr">
+        <is>
+          <t>อัตราไหล (m³/s ที่ 40 °C) × ความดันตก ÷ ประสิทธิภาพ</t>
+        </is>
+      </c>
+      <c r="I24" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต + ค่าด้านบน</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มน้ำหอทำเย็น</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C25" s="44" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D25" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E25" s="42">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="42">
+        <f>E25*$B$5</f>
+        <v/>
+      </c>
+      <c r="G25" s="43">
+        <f>E25/$E$43</f>
+        <v/>
+      </c>
+      <c r="H25" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ – ต้องรู้อุณหภูมิควันและภาระทำเย็น</t>
+        </is>
+      </c>
+      <c r="I25" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊ม MEA (2 ตัว รวม)</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="C26" s="41">
+        <f>2*'ขนาดการผลิต'!B16/3600/$B$11*$B$11*9.81*$B$9/$B$10/1000</f>
+        <v/>
+      </c>
+      <c r="D26" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E26" s="42">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="42">
+        <f>E26*$B$5</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>E26/$E$43</f>
+        <v/>
+      </c>
+      <c r="H26" s="31" t="inlineStr">
+        <is>
+          <t>2 × อัตราไหล × ρ g h ÷ ประสิทธิภาพ</t>
+        </is>
+      </c>
+      <c r="I26" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต + ค่าด้านบน</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มน้ำหล่อเย็น (ทำเย็น MEA + ควบแน่น)</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="C27" s="44" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D27" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E27" s="42">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="42">
+        <f>E27*$B$5</f>
+        <v/>
+      </c>
+      <c r="G27" s="43">
+        <f>E27/$E$43</f>
+        <v/>
+      </c>
+      <c r="H27" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I27" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>เครื่องวัด CO₂ (NDIR)</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="C28" s="44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D28" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E28" s="42">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="42">
+        <f>E28*$B$5</f>
+        <v/>
+      </c>
+      <c r="G28" s="43">
+        <f>E28/$E$43</f>
+        <v/>
+      </c>
+      <c r="H28" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I28" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>เครื่องอัด CO₂ 1.5→50 bar</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="C29" s="41">
+        <f>$B$14*$B$15/($B$15-1)*8.314*$B$19/0.04401*(($B$13/$B$12)^(($B$15-1)/($B$15*$B$14))-1)/$B$20*'ขนาดการผลิต'!B14/3600/1000</f>
+        <v/>
+      </c>
+      <c r="D29" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E29" s="42">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="42">
+        <f>E29*$B$5</f>
+        <v/>
+      </c>
+      <c r="G29" s="43">
+        <f>E29/$E$43</f>
+        <v/>
+      </c>
+      <c r="H29" s="31" t="inlineStr">
+        <is>
+          <t>สูตรอัดก๊าซหลายขั้น ทำเย็นระหว่างขั้น × อัตราไหล CO₂</t>
+        </is>
+      </c>
+      <c r="I29" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต + ค่าด้านบน</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>PEM ผลิต H₂</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C30" s="41">
+        <f>'ขนาดการผลิต'!B3</f>
+        <v/>
+      </c>
+      <c r="D30" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E30" s="42">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="42">
+        <f>E30*$B$5</f>
+        <v/>
+      </c>
+      <c r="G30" s="43">
+        <f>E30/$E$43</f>
+        <v/>
+      </c>
+      <c r="H30" s="31" t="inlineStr">
+        <is>
+          <t>กำลังตามสเปก (ใช้ 51.2 kWh/kg H₂, S09)</t>
+        </is>
+      </c>
+      <c r="I30" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม + S09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>ระบบกรองน้ำ RO/DI</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="C31" s="44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E31" s="42">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="42">
+        <f>E31*$B$5</f>
+        <v/>
+      </c>
+      <c r="G31" s="43">
+        <f>E31/$E$43</f>
+        <v/>
+      </c>
+      <c r="H31" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I31" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>H₂ Deoxo &amp; Dryer</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="C32" s="44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D32" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E32" s="42">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="42">
+        <f>E32*$B$5</f>
+        <v/>
+      </c>
+      <c r="G32" s="43">
+        <f>E32/$E$43</f>
+        <v/>
+      </c>
+      <c r="H32" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I32" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>เครื่องอัด H₂ 30→50 bar</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C33" s="41">
+        <f>1*$B$18/($B$18-1)*8.314*$B$19/0.002016*(($B$17/$B$16)^(($B$18-1)/($B$18*1))-1)/$B$20*'ขนาดการผลิต'!B12/3600/1000</f>
+        <v/>
+      </c>
+      <c r="D33" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E33" s="42">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="42">
+        <f>E33*$B$5</f>
+        <v/>
+      </c>
+      <c r="G33" s="43">
+        <f>E33/$E$43</f>
+        <v/>
+      </c>
+      <c r="H33" s="31" t="inlineStr">
+        <is>
+          <t>สูตรอัดก๊าซ 1 ขั้น × อัตราไหล H₂</t>
+        </is>
+      </c>
+      <c r="I33" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต + ค่าด้านบน</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>ใบกวนเตาปฏิกรณ์</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D34" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E34" s="42">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="42">
+        <f>E34*$B$5</f>
+        <v/>
+      </c>
+      <c r="G34" s="43">
+        <f>E34/$E$43</f>
+        <v/>
+      </c>
+      <c r="H34" s="31" t="inlineStr">
+        <is>
+          <t>กำลังพิกัดตามสเปก (ใช้จริงอาจน้อยกว่า)</t>
+        </is>
+      </c>
+      <c r="I34" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มป้อนตัวเร่ง/เอมีน</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="C35" s="44" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D35" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E35" s="42">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="42">
+        <f>E35*$B$5</f>
+        <v/>
+      </c>
+      <c r="G35" s="43">
+        <f>E35/$E$43</f>
+        <v/>
+      </c>
+      <c r="H35" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I35" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มสุญญากาศหอแยก</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="C36" s="44" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D36" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E36" s="42">
+        <f>C36*D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="42">
+        <f>E36*$B$5</f>
+        <v/>
+      </c>
+      <c r="G36" s="43">
+        <f>E36/$E$43</f>
+        <v/>
+      </c>
+      <c r="H36" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I36" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Chiller ควบแน่นกรด</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="C37" s="41">
+        <f>30/$B$21</f>
+        <v/>
+      </c>
+      <c r="D37" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E37" s="42">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="42">
+        <f>E37*$B$5</f>
+        <v/>
+      </c>
+      <c r="G37" s="43">
+        <f>E37/$E$43</f>
+        <v/>
+      </c>
+      <c r="H37" s="31" t="inlineStr">
+        <is>
+          <t>ความเย็น 30 kW (สเปกทีม) ÷ COP</t>
+        </is>
+      </c>
+      <c r="I37" s="31" t="inlineStr">
+        <is>
+          <t>ไฟล์ทีม + COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มหมุนเวียนเอมีน</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="C38" s="44" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D38" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E38" s="42">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="42">
+        <f>E38*$B$5</f>
+        <v/>
+      </c>
+      <c r="G38" s="43">
+        <f>E38/$E$43</f>
+        <v/>
+      </c>
+      <c r="H38" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I38" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>Scrubber ไอกรด</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="C39" s="44" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D39" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E39" s="42">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="42">
+        <f>E39*$B$5</f>
+        <v/>
+      </c>
+      <c r="G39" s="43">
+        <f>E39/$E$43</f>
+        <v/>
+      </c>
+      <c r="H39" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I39" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>ปั๊มถ่ายกรด (ใช้วันละ ~1 ชม.)</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="C40" s="44" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D40" s="40" t="n">
+        <v>365</v>
+      </c>
+      <c r="E40" s="42">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="42">
+        <f>E40*$B$5</f>
+        <v/>
+      </c>
+      <c r="G40" s="43">
+        <f>E40/$E$43</f>
+        <v/>
+      </c>
+      <c r="H40" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+      <c r="I40" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>PLC + เซนเซอร์ + IoT</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>5.x</t>
+        </is>
+      </c>
+      <c r="C41" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="40" t="n">
+        <v>8760</v>
+      </c>
+      <c r="E41" s="42">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="42">
+        <f>E41*$B$5</f>
+        <v/>
+      </c>
+      <c r="G41" s="43">
+        <f>E41/$E$43</f>
+        <v/>
+      </c>
+      <c r="H41" s="31" t="inlineStr">
+        <is>
+          <t>เปิดตลอดปี</t>
+        </is>
+      </c>
+      <c r="I41" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>ไฟส่องสว่าง/อื่น ๆ ใน skid</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t>6.x</t>
+        </is>
+      </c>
+      <c r="C42" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="40" t="n">
+        <v>8760</v>
+      </c>
+      <c r="E42" s="42">
+        <f>C42*D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="42">
+        <f>E42*$B$5</f>
+        <v/>
+      </c>
+      <c r="G42" s="43">
+        <f>E42/$E$43</f>
+        <v/>
+      </c>
+      <c r="H42" s="31" t="inlineStr">
+        <is>
+          <t>เปิดตลอดปี</t>
+        </is>
+      </c>
+      <c r="I42" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="45" t="inlineStr">
+        <is>
+          <t>รวมไฟฟ้าทั้งหมด</t>
+        </is>
+      </c>
+      <c r="C43" s="46">
+        <f>SUM(C24:C42)</f>
+        <v/>
+      </c>
+      <c r="E43" s="47">
+        <f>SUM(E24:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="47">
+        <f>SUM(F24:F42)</f>
+        <v/>
+      </c>
+      <c r="G43" s="48">
+        <f>SUM(G24:G42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>ความร้อน (ไอน้ำ) – ไม่ใช่ไฟฟ้า</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>รายการ</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>กำลังความร้อน (kW)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>ชั่วโมง/ปี</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>GJ/ปี</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>ค่าไอน้ำ (บาท/ปี)</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>ราคาไอน้ำ (บาท/GJ)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>วิธีคำนวณ</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>ที่มา</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="29" t="inlineStr">
+        <is>
+          <t>หม้อต้มหอไล่ CO₂</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="C48" s="32">
+        <f>'ขนาดการผลิต'!B17</f>
+        <v/>
+      </c>
+      <c r="D48" s="30">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E48" s="42">
+        <f>C48*D48*3.6/1000</f>
+        <v/>
+      </c>
+      <c r="F48" s="42">
+        <f>E48*G48</f>
+        <v/>
+      </c>
+      <c r="G48" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="31" t="inlineStr">
+        <is>
+          <t>CO₂ kg/ชม. × 3.7 GJ/t (S06); ราคา 0 = ใช้ไอน้ำเหลือทิ้งฟรี ต้องตกลงกับ กฟผ.</t>
+        </is>
+      </c>
+      <c r="I48" s="31" t="inlineStr">
+        <is>
+          <t>S06 + ชีต ขนาดการผลิต</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="29" t="inlineStr">
+        <is>
+          <t>หม้อต้มหอแยกกรด (3.5)</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>ยังไม่ทราบ</t>
+        </is>
+      </c>
+      <c r="H49" s="31" t="inlineStr">
+        <is>
+          <t>ต้องดูจากตารางเสริม S16–S19 ของงาน Tzitzili หรือผู้ขาย</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ค่าดำเนินการและระยะคืนทุน (Skid 100 kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>คืนทุนแบบง่าย = เงินลงทุน ÷ กำไรต่อปี (ยังไม่รวมภาษี ดอกเบี้ย ค่าเช่าพื้นที่)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>รายการ</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ค่า</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>หน่วย</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ที่มา</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>เงินลงทุนรวม</t>
+        </is>
+      </c>
+      <c r="B5" s="30">
+        <f>'งบลงทุน'!F71</f>
+        <v/>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>บาท</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>ชีต งบลงทุน</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>ผลผลิตกรด 85%</t>
+        </is>
+      </c>
+      <c r="B6" s="32">
+        <f>'ขนาดการผลิต'!B19</f>
+        <v/>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ใช้</t>
+        </is>
+      </c>
+      <c r="B7" s="32">
+        <f>'ขนาดการผลิต'!B14*'ขนาดการผลิต'!B5/1000</f>
+        <v/>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>ค่าไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="B8" s="30">
+        <f>'การใช้ไฟ'!F43</f>
+        <v/>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>ชีต การใช้ไฟ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>ค่าไอน้ำ</t>
+        </is>
+      </c>
+      <c r="B9" s="30">
+        <f>'การใช้ไฟ'!F48</f>
+        <v/>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>ชีต การใช้ไฟ (ค่าเริ่ม 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>ซ่อมบำรุงต่อปี (% ของเงินลงทุน)</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ – ค่าทั่วไป 2–4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>ค่าซ่อมบำรุง</t>
+        </is>
+      </c>
+      <c r="B11" s="42">
+        <f>$B$5*$B$10</f>
+        <v/>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>จำนวนช่างเดินเครื่อง</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>คน</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>เงินเดือน</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>บาท/เดือน</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>ค่าแรง (13 เดือน)</t>
+        </is>
+      </c>
+      <c r="B14" s="42">
+        <f>$B$12*$B$13*13</f>
+        <v/>
+      </c>
+      <c r="C14" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>ราคา MEA</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="n">
+        <v>60</v>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>บาท/กก.</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ – ต้องขอใบเสนอราคา</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>MEA เติมชดเชย</t>
+        </is>
+      </c>
+      <c r="B16" s="42">
+        <f>$B$7*2.2*$B$15</f>
+        <v/>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>2.2 กก./ตัน CO₂ (S07) × ราคา</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>เอมีน + ตัวเร่ง Ru เติมชดเชย</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>400000</v>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>ประมาณการ – ต้องขอข้อมูล</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>รวมค่าดำเนินการ</t>
+        </is>
+      </c>
+      <c r="B18" s="50">
+        <f>$B$8+$B$9+$B$11+$B$14+$B$16+$B$17</f>
+        <v/>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>บาท/ปี</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ราคาขาย</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>30 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>39.78 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>52.3 บาท/กก.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>ราคาขาย (บาท/กก. กรด 85%)</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="C21" s="35" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="D21" s="35" t="n">
+        <v>52.3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>ที่มาราคา</t>
+        </is>
+      </c>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>สมมติ: ต้องขายถูกกว่าราคานำเข้ามาก</t>
+        </is>
+      </c>
+      <c r="C22" s="51" t="inlineStr">
+        <is>
+          <t>S11 ราคาในงาน Tzitzili 1.40 USD/kg × 0.85 × 33.426</t>
+        </is>
+      </c>
+      <c r="D22" s="51" t="inlineStr">
+        <is>
+          <t>S15 ราคายกลังที่เกษตรกรจ่าย (สูงเกินจริงสำหรับขายผู้นำเข้า)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>รายได้ (บาท/ปี)</t>
+        </is>
+      </c>
+      <c r="B23" s="42">
+        <f>$B$6*1000*B21</f>
+        <v/>
+      </c>
+      <c r="C23" s="42">
+        <f>$B$6*1000*C21</f>
+        <v/>
+      </c>
+      <c r="D23" s="42">
+        <f>$B$6*1000*D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>ค่าดำเนินการ (บาท/ปี)</t>
+        </is>
+      </c>
+      <c r="B24" s="42">
+        <f>$B$18</f>
+        <v/>
+      </c>
+      <c r="C24" s="42">
+        <f>$B$18</f>
+        <v/>
+      </c>
+      <c r="D24" s="42">
+        <f>$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>กำไรก่อนภาษี (บาท/ปี)</t>
+        </is>
+      </c>
+      <c r="B25" s="53">
+        <f>B23-B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="53">
+        <f>C23-C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="53">
+        <f>D23-D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="45" t="inlineStr">
+        <is>
+          <t>ระยะคืนทุน (ปี)</t>
+        </is>
+      </c>
+      <c r="B26" s="54">
+        <f>IF(B25&gt;0,$B$5/B25,"ไม่คืนทุน")</f>
+        <v/>
+      </c>
+      <c r="C26" s="54">
+        <f>IF(C25&gt;0,$B$5/C25,"ไม่คืนทุน")</f>
+        <v/>
+      </c>
+      <c r="D26" s="54">
+        <f>IF(D25&gt;0,$B$5/D25,"ไม่คืนทุน")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>กระแสเงินสดสะสม (บาท)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>ปีที่</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>30 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>39.78 บาท/กก.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>52.3 บาท/กก.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="B30" s="42">
+        <f>-$B$5</f>
+        <v/>
+      </c>
+      <c r="C30" s="42">
+        <f>-$B$5</f>
+        <v/>
+      </c>
+      <c r="D30" s="42">
+        <f>-$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="42">
+        <f>B30+B$25</f>
+        <v/>
+      </c>
+      <c r="C31" s="42">
+        <f>C30+C$25</f>
+        <v/>
+      </c>
+      <c r="D31" s="42">
+        <f>D30+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="42">
+        <f>B31+B$25</f>
+        <v/>
+      </c>
+      <c r="C32" s="42">
+        <f>C31+C$25</f>
+        <v/>
+      </c>
+      <c r="D32" s="42">
+        <f>D31+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="42">
+        <f>B32+B$25</f>
+        <v/>
+      </c>
+      <c r="C33" s="42">
+        <f>C32+C$25</f>
+        <v/>
+      </c>
+      <c r="D33" s="42">
+        <f>D32+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" s="42">
+        <f>B33+B$25</f>
+        <v/>
+      </c>
+      <c r="C34" s="42">
+        <f>C33+C$25</f>
+        <v/>
+      </c>
+      <c r="D34" s="42">
+        <f>D33+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" s="42">
+        <f>B34+B$25</f>
+        <v/>
+      </c>
+      <c r="C35" s="42">
+        <f>C34+C$25</f>
+        <v/>
+      </c>
+      <c r="D35" s="42">
+        <f>D34+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" s="42">
+        <f>B35+B$25</f>
+        <v/>
+      </c>
+      <c r="C36" s="42">
+        <f>C35+C$25</f>
+        <v/>
+      </c>
+      <c r="D36" s="42">
+        <f>D35+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="55" t="n">
+        <v>7</v>
+      </c>
+      <c r="B37" s="42">
+        <f>B36+B$25</f>
+        <v/>
+      </c>
+      <c r="C37" s="42">
+        <f>C36+C$25</f>
+        <v/>
+      </c>
+      <c r="D37" s="42">
+        <f>D36+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="B38" s="42">
+        <f>B37+B$25</f>
+        <v/>
+      </c>
+      <c r="C38" s="42">
+        <f>C37+C$25</f>
+        <v/>
+      </c>
+      <c r="D38" s="42">
+        <f>D37+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="B39" s="42">
+        <f>B38+B$25</f>
+        <v/>
+      </c>
+      <c r="C39" s="42">
+        <f>C38+C$25</f>
+        <v/>
+      </c>
+      <c r="D39" s="42">
+        <f>D38+D$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="B40" s="42">
+        <f>B39+B$25</f>
+        <v/>
+      </c>
+      <c r="C40" s="42">
+        <f>C39+C$25</f>
+        <v/>
+      </c>
+      <c r="D40" s="42">
+        <f>D39+D$25</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ดักจับและลดได้สุทธิ (Skid 100 kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>รายการ</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ค่า</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>หน่วย</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ที่มา</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ดักจับและใช้ผลิตกรด</t>
+        </is>
+      </c>
+      <c r="B4" s="32">
+        <f>'ขนาดการผลิต'!B14*'ขนาดการผลิต'!B5/1000</f>
+        <v/>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>ชีต ขนาดการผลิต</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ จากไฟโรงไฟฟ้าบางปะกง</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/MWh</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>4.55 Mt ÷ 12.2 TWh (S02 + S04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า PEM</t>
+        </is>
+      </c>
+      <c r="B6" s="32">
+        <f>'การใช้ไฟ'!E30/1000</f>
+        <v/>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>MWh/ปี</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="inlineStr">
+        <is>
+          <t>ชีต การใช้ไฟ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>ไฟฟ้าอุปกรณ์อื่น</t>
+        </is>
+      </c>
+      <c r="B7" s="57">
+        <f>'การใช้ไฟ'!E43/1000-B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>MWh/ปี</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
+        <is>
+          <t>ชีต การใช้ไฟ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>CO₂ ที่บางปะกงปล่อยทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="n">
+        <v>4550000</v>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>ตัน/ปี</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>bang_pakong_co2.py (S02 + S04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>กรณีแหล่งไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>CO₂ จากการใช้ไฟ (ตัน/ปี)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ลดสุทธิ (ตัน/ปี)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>% ของ CO₂ บางปะกง</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>ไฟจากโรงไฟฟ้าก๊าซทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B11" s="57">
+        <f>($B$6+$B$7)*$B$5</f>
+        <v/>
+      </c>
+      <c r="C11" s="58">
+        <f>$B$4-B11</f>
+        <v/>
+      </c>
+      <c r="D11" s="59">
+        <f>C11/$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>PEM ใช้โซลาร์, อุปกรณ์อื่นใช้ไฟโรงไฟฟ้า</t>
+        </is>
+      </c>
+      <c r="B12" s="57">
+        <f>$B$7*$B$5</f>
+        <v/>
+      </c>
+      <c r="C12" s="58">
+        <f>$B$4-B12</f>
+        <v/>
+      </c>
+      <c r="D12" s="59">
+        <f>C12/$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>ใช้โซลาร์ทั้งหมด</t>
+        </is>
+      </c>
+      <c r="B13" s="57">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C13" s="58">
+        <f>$B$4-B13</f>
+        <v/>
+      </c>
+      <c r="D13" s="59">
+        <f>C13/$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>CO₂ ที่ลดได้นอกบางปะกง (แทนกรดนำเข้า)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>กรดแบบเดิม (ตัน CO₂e ต่อตันกรด)</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>S20 Cuevas-Castillo et al. 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>กรดจาก CO₂ (ตัน CO₂e ต่อตันกรด)</t>
+        </is>
+      </c>
+      <c r="B17" s="56" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>ลดได้จากการแทนกรดนำเข้า (ตัน CO₂e/ปี)</t>
+        </is>
+      </c>
+      <c r="B18" s="58">
+        <f>'ขนาดการผลิต'!B18*(B16-B17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>เกิดที่ประเทศผู้ผลิตกรด ไม่ใช่ที่บางปะกง</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>